<commit_message>
FOVI2026: retira a C. Díaz, M. Macaya y UCM; red de cinco instituciones
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P4g3Yf3jcPuX77QSmk15pC
</commit_message>
<xml_diff>
--- a/fovi2026/final/FOVI2026_Presupuesto-carta-gantt_FINAL.xlsx
+++ b/fovi2026/final/FOVI2026_Presupuesto-carta-gantt_FINAL.xlsx
@@ -2106,7 +2106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q102"/>
+  <dimension ref="B2:Q102"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15"/>
   <cols>
     <col width="2.7109375" customWidth="1" min="1" max="1"/>
@@ -2116,7 +2116,6 @@
     <col width="4.5703125" customWidth="1" min="6" max="17"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="39.75" customHeight="1">
       <c r="B2" s="182" t="inlineStr">
         <is>
@@ -2369,7 +2368,7 @@
     <row r="11">
       <c r="B11" s="189" t="inlineStr">
         <is>
-          <t>Objetivo 1 (OE1): Formalizar y activar la red USACH–UCM–UJPA–UPCoimbra–UNESPAR–UNILAB</t>
+          <t>Objetivo 1 (OE1): Formalizar y activar la red USACH–UJPA–UPCoimbra–UNESPAR–UNILAB</t>
         </is>
       </c>
       <c r="C11" s="190" t="inlineStr">
@@ -4604,7 +4603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="B2:I48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="9.140625" customWidth="1" style="13" min="1" max="2"/>
@@ -5451,7 +5450,6 @@
       <c r="H42" s="34" t="n"/>
       <c r="I42" s="35" t="n"/>
     </row>
-    <row r="43"/>
     <row r="44" ht="15.75" customHeight="1">
       <c r="B44" s="36" t="inlineStr">
         <is>
@@ -5531,7 +5529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S82"/>
+  <dimension ref="B2:S82"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="11.42578125" customWidth="1" style="76" min="1" max="1"/>
@@ -5544,7 +5542,6 @@
     <col width="11.42578125" customWidth="1" style="76" min="8" max="14"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="80" t="inlineStr">
         <is>
@@ -5552,7 +5549,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="80" t="inlineStr">
         <is>
@@ -5995,7 +5991,7 @@
       </c>
       <c r="D23" s="235" t="inlineStr">
         <is>
-          <t>Actividad 5. Pasantía en Coimbra (ISEC-UPCoimbra, Portugal): 2 integrantes del grupo chileno (1 USACH, 1 UCM). 2 pasajes aéreos económicos Santiago–Coimbra (vía Lisboa/Porto), ida y vuelta, punto a punto, 2 × $1.500.000. ESTIMACIÓN: cotizar antes de enviar.</t>
+          <t>Actividad 5. Pasantía en Coimbra (ISEC-UPCoimbra, Portugal): 2 integrantes del grupo chileno (USACH). 2 pasajes aéreos económicos Santiago–Coimbra (vía Lisboa/Porto), ida y vuelta, punto a punto, 2 × $1.500.000. ESTIMACIÓN: cotizar antes de enviar.</t>
         </is>
       </c>
       <c r="H23" s="231" t="n"/>
@@ -6019,7 +6015,7 @@
       </c>
       <c r="D24" s="236" t="inlineStr">
         <is>
-          <t>Actividad 6. Pasantía en Luanda (UJPA, Angola): 2 integrantes del grupo chileno (USACH y UCM). 2 pasajes aéreos económicos Santiago–Luanda, ida y vuelta, 2 × $2.500.000. ESTIMACIÓN: cotizar antes de enviar.</t>
+          <t>Actividad 6. Pasantía en Luanda (UJPA, Angola): 2 integrantes del grupo chileno (USACH). 2 pasajes aéreos económicos Santiago–Luanda, ida y vuelta, 2 × $2.500.000. ESTIMACIÓN: cotizar antes de enviar.</t>
         </is>
       </c>
       <c r="H24" s="231" t="n"/>
@@ -6556,7 +6552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S84"/>
+  <dimension ref="B2:S84"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="29.42578125" customWidth="1" min="2" max="2"/>
@@ -6566,7 +6562,6 @@
     <col width="10" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="49" t="inlineStr">
         <is>
@@ -6574,7 +6569,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="80" t="inlineStr">
         <is>
@@ -7434,7 +7428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S79"/>
+  <dimension ref="B2:S79"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="29.42578125" customWidth="1" min="2" max="2"/>
@@ -7443,7 +7437,6 @@
     <col width="21.140625" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="49" t="inlineStr">
         <is>
@@ -7451,7 +7444,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="80" t="inlineStr">
         <is>
@@ -8259,7 +8251,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="B2:E32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="11.42578125" customWidth="1" min="1" max="1"/>
@@ -8269,7 +8261,6 @@
     <col width="25" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="32.25" customHeight="1">
       <c r="B2" s="181" t="inlineStr">
         <is>

</xml_diff>